<commit_message>
제목에 GitHub Pages 링크 추가 2026-05-19
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260519.xlsx
+++ b/RNR_수입원가_2026_20260519.xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0&quot;일&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="맑은 고딕"/>
       <charset val="129"/>
@@ -184,6 +184,13 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="17">
@@ -419,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="206">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1009,6 +1016,9 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1414,9 +1424,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="169" t="inlineStr">
-        <is>
-          <t>RNR 2026년 PO별 수입원가 산출표 (Master)</t>
+      <c r="A1" s="206" t="inlineStr">
+        <is>
+          <t>RNR 2026년 PO별 수입원가 산출표 (Master)  📊 https://rnrfin.github.io/rnr-importcost/</t>
         </is>
       </c>
       <c r="B1" s="148" t="n"/>
@@ -9225,6 +9235,9 @@
     <mergeCell ref="O3:W3"/>
     <mergeCell ref="A2:AF2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -15102,7 +15115,6 @@
         <v/>
       </c>
     </row>
-    <row r="75"/>
     <row r="76">
       <c r="M76" s="40" t="n"/>
     </row>

</xml_diff>